<commit_message>
Added Impact Drilldown, Event Roster, and Export Names
</commit_message>
<xml_diff>
--- a/Context Data/2024 - 2025 MASTER.ROSTER (version 1).xlsx
+++ b/Context Data/2024 - 2025 MASTER.ROSTER (version 1).xlsx
@@ -15400,9 +15400,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B4ED48AFA98C9D4CBDAB85A9D631CF97" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e58c25bcd981d8c8d65677a9b5215e90">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="603e6958-f347-4390-937b-f81c7f882348" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3c75a39d0b2707d4d405c626d1715ccf" ns2:_="">
-    <xsd:import namespace="603e6958-f347-4390-937b-f81c7f882348"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D9425BFD98FC2C4FA733E6DF42251950" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="495a1111c3181cda2ad14b2e0945a813">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fff059bb-b667-4476-9a60-571bf927bc8d" xmlns:ns3="dfeb989f-b0e3-4d2a-bb54-484d4dc74e52" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bba7d42f9d6e23798750fbd8095ac435" ns2:_="" ns3:_="">
+    <xsd:import namespace="fff059bb-b667-4476-9a60-571bf927bc8d"/>
+    <xsd:import namespace="dfeb989f-b0e3-4d2a-bb54-484d4dc74e52"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -15416,6 +15417,10 @@
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -15423,7 +15428,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="603e6958-f347-4390-937b-f81c7f882348" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="fff059bb-b667-4476-9a60-571bf927bc8d" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -15460,6 +15465,40 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="138fa7a7-b18c-4352-a067-90bbe88a6642" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="dfeb989f-b0e3-4d2a-bb54-484d4dc74e52" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{ed739e65-922e-410f-a9ab-5ebaf558b2b6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="dfeb989f-b0e3-4d2a-bb54-484d4dc74e52">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -15572,12 +15611,17 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="dfeb989f-b0e3-4d2a-bb54-484d4dc74e52" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fff059bb-b667-4476-9a60-571bf927bc8d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D1C723B-2A49-4BE0-A198-5A71E009D93C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7E24251-3AAE-42F0-9B99-3EF2033FC265}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>